<commit_message>
push task week 4 and update testcases
</commit_message>
<xml_diff>
--- a/Extra/TC/Test Cases.xlsx
+++ b/Extra/TC/Test Cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhuan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UTH mãi đỉnh\Lập trình Mạng\Project\NET_09-CO-TUONG\Extra\TC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5710C47E-D8B7-4933-A999-6F187FD287F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF4CDF5-477E-4C2F-9D28-89A63DE9FC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,9 +23,21 @@
     <sheet name="TC_07" sheetId="8" r:id="rId8"/>
     <sheet name="TC_08" sheetId="9" r:id="rId9"/>
     <sheet name="TC_09" sheetId="10" r:id="rId10"/>
+    <sheet name="TC_10" sheetId="13" r:id="rId11"/>
+    <sheet name="TC_11" sheetId="14" r:id="rId12"/>
+    <sheet name="TC_12" sheetId="15" r:id="rId13"/>
+    <sheet name="TC_13" sheetId="16" r:id="rId14"/>
+    <sheet name="TC_14" sheetId="17" r:id="rId15"/>
+    <sheet name="TC_15" sheetId="18" r:id="rId16"/>
+    <sheet name="TC_16" sheetId="19" r:id="rId17"/>
+    <sheet name="TC_17" sheetId="20" r:id="rId18"/>
+    <sheet name="TC_18" sheetId="21" r:id="rId19"/>
+    <sheet name="TC_19" sheetId="22" r:id="rId20"/>
+    <sheet name="TC_20" sheetId="11" r:id="rId21"/>
+    <sheet name="TC_21" sheetId="12" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="Z_594E70F7_1077_448A_A0CF_FD3289E530C0_.wvu.FilterData" localSheetId="0" hidden="1">'Danh Sách Test_Case'!$B$2:$K$13</definedName>
+    <definedName name="Z_594E70F7_1077_448A_A0CF_FD3289E530C0_.wvu.FilterData" localSheetId="0" hidden="1">'Danh Sách Test_Case'!$B$2:$K$23</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <customWorkbookViews>
@@ -33,14 +45,14 @@
   </customWorkbookViews>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId11" roundtripDataChecksum="hICAFeWSzinCYtVsJX+hRSQRkFPchBtuGo4dofo2yYo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId23" roundtripDataChecksum="hICAFeWSzinCYtVsJX+hRSQRkFPchBtuGo4dofo2yYo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="125">
   <si>
     <t>TC_01</t>
   </si>
@@ -252,12 +264,229 @@
 Server gửi thông báo đến Client 2.
 Client 2 hiện trong khung chat: [Game] Đối thủ đã thoát khỏi phòng. và chuyển cờ về offline (_isOnline = false).</t>
   </si>
+  <si>
+    <t>TC_10</t>
+  </si>
+  <si>
+    <t>TC_11</t>
+  </si>
+  <si>
+    <t>TC_12</t>
+  </si>
+  <si>
+    <t>TC_13</t>
+  </si>
+  <si>
+    <t>TC_14</t>
+  </si>
+  <si>
+    <t>TC_15</t>
+  </si>
+  <si>
+    <t>TC_16</t>
+  </si>
+  <si>
+    <t>TC_17</t>
+  </si>
+  <si>
+    <t>TC_18</t>
+  </si>
+  <si>
+    <t>TC_19</t>
+  </si>
+  <si>
+    <t>TC_10!A1</t>
+  </si>
+  <si>
+    <t>MoveValidator - Tướng</t>
+  </si>
+  <si>
+    <t>Kiểm tra luật đi của quân Tướng (trong cung, 1 ô ngang/dọc)</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Ván cờ đang chạy, Tướng Đỏ ở vị trí (4, 9).
+Thao tác:
+1. Thử đi Tướng lên 1 ô (4, 8).
+2. Thử đi Tướng chéo hoặc đi ra ngoài cung (ví dụ ra cột 2).</t>
+  </si>
+  <si>
+    <t>Đi thẳng 1 ô trong cung: Thành công.
+Đi chéo hoặc ra ngoài phạm vi cung (cột 3-5, hàng 7-9): Bị chặn, quân Tướng không di</t>
+  </si>
+  <si>
+    <t>Đúng như mong đợi</t>
+  </si>
+  <si>
+    <t>MoveValidator - Sĩ</t>
+  </si>
+  <si>
+    <t>Kiểm tra luật đi chéo trong cung của quân Sĩ</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Sĩ Đỏ ở vị trí (3, 9).
+Thao tác:
+1. Click Sĩ và chọn ô tâm cung (4, 8).
+2. Từ (4, 8) thử đi ngang hoặc đi ra ngoài cung.</t>
+  </si>
+  <si>
+    <t>Đi chéo 1 bước trong cung: Hợp lệ.
+Đi thẳng hoặc ra ngoài cung: Bị từ chối, không đi được.</t>
+  </si>
+  <si>
+    <t>MoveValidator - Tượng</t>
+  </si>
+  <si>
+    <t>Kiểm tra Tượng đi chéo 2 ô, không qua sông và bị cản mắt Tượng</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Tượng Đỏ ở (2, 9).
+Thao tác:
+1. Cho 1 quân khác đứng ở tâm chéo (3, 8) rồi thử đi Tượng đến (4, 7).
+2. Đưa Tượng lên bờ sông và thử nhảy sang phần sân bên kia (qua sông).</t>
+  </si>
+  <si>
+    <t>Khi bị cản mắt: Không đi được.
+Thử nhảy qua sông: Bị chặn, Tượng chỉ được ở sân nhà.</t>
+  </si>
+  <si>
+    <t>MoveValidator - Mã</t>
+  </si>
+  <si>
+    <t>Kiểm tra Mã đi chữ L và bắt lỗi cản chân Mã</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Mã Đỏ ở (1, 9), phía trước có quân đứng tại (1, 8) (bị cản chân dọc).
+Thao tác:
+1. Cố tình chọn Mã và click ô (2, 7) khi chân bị cản.
+2. Mở đường (di chuyển quân cản đi chỗ khác) rồi đi lại.</t>
+  </si>
+  <si>
+    <t>Khi có quân cản chân: Không di chuyển được.
+Khi chân Mã thông: Đi chữ L thành công đến ô đích, phát âm thanh di chuyển.</t>
+  </si>
+  <si>
+    <t>MoveValidator - Xe</t>
+  </si>
+  <si>
+    <t>Kiểm tra Xe đi ngang/dọc không giới hạn và không được nhảy quân</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Xe Đỏ ở (0, 9).
+Thao tác:
+1. Thử đi Xe xuyên qua quân Tốt của mình ở hàng trên.
+2. Đi Xe trên đường thẳng không có vật cản và ăn 1 quân địch ở cuối đường.</t>
+  </si>
+  <si>
+    <t>Không được nhảy qua quân cản trên đường đi.
+Đi thẳng hoặc ăn quân đối phương nếu đường đi thông suốt.</t>
+  </si>
+  <si>
+    <t>MoveValidator - Pháo</t>
+  </si>
+  <si>
+    <t>Kiểm tra Pháo đi thông thường và luật ăn quân cần đúng 1 ngòi</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Pháo Đỏ ở (1, 7).
+Thao tác:
+1. Đi Pháo vào ô trống thẳng hàng không có quân cản.
+2. Nhảy qua đúng 1 quân bất kỳ để ăn quân địch phía sau.
+3. Thử ăn quân địch khi ở giữa có 0 quân hoặc 2 quân làm ngòi.</t>
+  </si>
+  <si>
+    <t>Đi ô trống: Hợp lệ nếu đường thông.
+Ăn quân có đúng 1 ngòi: Thành công.
+Ăn quân khi có 0 hoặc ≥2 ngòi: Bị từ chối.[@[Name/Screen]]</t>
+  </si>
+  <si>
+    <t>MoveValidator - Tốt</t>
+  </si>
+  <si>
+    <t>Kiểm tra Tốt trước và sau khi qua sông</t>
+  </si>
+  <si>
+    <t>Ngữ cảnh: Tốt Đỏ tại vị trí xuất phát (4, 6).
+Thao tác:
+1. Lúc chưa qua sông: Thử đi ngang hoặc lùi.
+2. Đi thẳng tiến qua sông: Thử đi ngang và đi thẳng. Thử đi lùi.</t>
+  </si>
+  <si>
+    <t>Chưa qua sông: Chỉ đi thẳng 1 bước; không đi ngang, không đi lùi.
+Đã qua sông: Được đi thẳng hoặc sang ngang 1 bước; tuyệt đối không được lùi.</t>
+  </si>
+  <si>
+    <t>TC_20</t>
+  </si>
+  <si>
+    <t>TC_21</t>
+  </si>
+  <si>
+    <t>TC_11!A1</t>
+  </si>
+  <si>
+    <t>TC_12!A1</t>
+  </si>
+  <si>
+    <t>TC_13!A1</t>
+  </si>
+  <si>
+    <t>TC_14!A1</t>
+  </si>
+  <si>
+    <t>TC_15!A1</t>
+  </si>
+  <si>
+    <t>TC_16!A1</t>
+  </si>
+  <si>
+    <t>TC_17!A1</t>
+  </si>
+  <si>
+    <t>TC_18!A1</t>
+  </si>
+  <si>
+    <t>TC_19!A1</t>
+  </si>
+  <si>
+    <t>ChatBox &amp; Result</t>
+  </si>
+  <si>
+    <t>Kiểm tra lệnh /surrender (Đầu hàng) và hiển thị kết quả trận đấu</t>
+  </si>
+  <si>
+    <t>Thao tác: Người chơi gõ lệnh /surrender vào ô chat và nhấn Enter.</t>
+  </si>
+  <si>
+    <t>Khung chat thông báo: Bạn đã đầu hàng!.
+Đối thủ nhận thông báo: Đối thủ đầu hàng! Bạn thắng!.
+Cả 2 bên xuất hiện bảng popup FormResult hiển thị Thắng/Thua tương ứng.@Test Result 1</t>
+  </si>
+  <si>
+    <t>Xử lý đầu hàng và kết thúc ván cờ chính xác qua Socket.</t>
+  </si>
+  <si>
+    <t>Mạng &amp; FormGame</t>
+  </si>
+  <si>
+    <t>Kiểm tra đồng bộ nước đi thời gian thực giữa 2 máy qua TCP</t>
+  </si>
+  <si>
+    <t>Tiền điều kiện: 2 Client đang trong phòng chơi, đến lượt Đỏ.
+Thao tác: Trên Client Đỏ, đi nước Pháo đầu từ (1, 7) sang (4, 7).</t>
+  </si>
+  <si>
+    <t>Client Đỏ: Quân Pháo dời sang (4, 7), đổi lượt sang Đen, reset timer.
+Client Đen: Nhận gói Move từ Server, quân Pháo của đối thủ tự động dời sang (4, 7), ô trạng thái chuyển sang Lượt Đen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nước đi cập nhật chính xác trên cả 2 màn hình, không bị trễ hay sai toạ độ.	</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,6 +546,11 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -553,22 +787,6 @@
       </fill>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor theme="0"/>
@@ -592,13 +810,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Danh Sách Test_Case-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="2"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="5"/>
+      <tableStyleElement type="headerRow" dxfId="4"/>
+      <tableStyleElement type="firstRowStripe" dxfId="3"/>
+      <tableStyleElement type="secondRowStripe" dxfId="2"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -650,6 +884,251 @@
         <a:xfrm>
           <a:off x="594360" y="350520"/>
           <a:ext cx="5867908" cy="594412"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>236822</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>69093</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{162D24FC-D694-B247-A672-9EB8EBE84B9B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6942422" cy="5921253"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>236822</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>107196</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E627FB2F-F8A2-0A11-017A-3A05A1901AE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6942422" cy="5959356"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>244442</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>69093</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E70090EE-B411-6F1F-DDEA-D922D3941067}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6950042" cy="5921253"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>16456</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>99576</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C24F0C37-2181-7902-4613-7C5CA9115DED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="14037256" cy="5951736"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>282546</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>130058</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35E2D733-1E53-DA5C-4C90-F01CD8B27343}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6988146" cy="5982218"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -857,8 +1336,204 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>252063</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>53852</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05887ED8-5EDB-7B35-C8CD-02A3162EE86E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6957663" cy="5906012"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>252063</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>152920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0C54163-5FCF-44C9-B564-0D8A48E438CB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6957663" cy="6005080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>244442</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>145300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{166C6BDB-7BEA-4855-B525-B6DF410E87D5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6950042" cy="5997460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>236822</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>76714</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7DB8C7C-1B96-26D2-7136-532E326E9A57}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="365760"/>
+          <a:ext cx="6942422" cy="5928874"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="B2:K13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="B2:K23">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name/Screen"/>
@@ -1073,13 +1748,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL1005"/>
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1:AL1015"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.109375" customWidth="1"/>
-    <col min="2" max="2" width="5.6640625" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" customWidth="1"/>
-    <col min="4" max="5" width="26.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.21875" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="37" customWidth="1"/>
     <col min="6" max="6" width="46.33203125" customWidth="1"/>
     <col min="7" max="7" width="27.5546875" customWidth="1"/>
     <col min="8" max="8" width="24.6640625" customWidth="1"/>
@@ -1368,7 +2047,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="121.2" customHeight="1">
+    <row r="6" spans="1:38" ht="138.6" customHeight="1">
       <c r="A6" s="2"/>
       <c r="B6" s="23" t="s">
         <v>20</v>
@@ -1424,7 +2103,7 @@
       <c r="AK6" s="2"/>
       <c r="AL6" s="2"/>
     </row>
-    <row r="7" spans="1:38" ht="79.8" customHeight="1">
+    <row r="7" spans="1:38" ht="100.2" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="23" t="s">
         <v>48</v>
@@ -1480,7 +2159,7 @@
       <c r="AK7" s="2"/>
       <c r="AL7" s="2"/>
     </row>
-    <row r="8" spans="1:38" ht="79.8" customHeight="1">
+    <row r="8" spans="1:38" ht="91.8" customHeight="1">
       <c r="A8" s="2"/>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -1536,19 +2215,31 @@
       <c r="AK8" s="2"/>
       <c r="AL8" s="2"/>
     </row>
-    <row r="9" spans="1:38" ht="79.8" customHeight="1">
+    <row r="9" spans="1:38" ht="135.6" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="16"/>
+      <c r="C9" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
-      <c r="J9" s="9"/>
+      <c r="J9" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="K9" s="18" t="s">
         <v>55</v>
       </c>
@@ -1585,14 +2276,26 @@
       <c r="B10" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="16"/>
+      <c r="C10" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
-      <c r="J10" s="9"/>
+      <c r="J10" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="K10" s="18" t="s">
         <v>57</v>
       </c>
@@ -1624,19 +2327,31 @@
       <c r="AK10" s="2"/>
       <c r="AL10" s="2"/>
     </row>
-    <row r="11" spans="1:38" ht="79.8" customHeight="1">
+    <row r="11" spans="1:38" ht="91.2" customHeight="1">
       <c r="A11" s="2"/>
       <c r="B11" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="16"/>
+      <c r="C11" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
-      <c r="J11" s="9"/>
+      <c r="J11" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="K11" s="18" t="s">
         <v>58</v>
       </c>
@@ -1668,19 +2383,31 @@
       <c r="AK11" s="2"/>
       <c r="AL11" s="2"/>
     </row>
-    <row r="12" spans="1:38" ht="79.8" customHeight="1">
+    <row r="12" spans="1:38" ht="108" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="16"/>
+      <c r="C12" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
-      <c r="J12" s="9"/>
+      <c r="J12" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="K12" s="18" t="s">
         <v>59</v>
       </c>
@@ -1712,20 +2439,34 @@
       <c r="AK12" s="2"/>
       <c r="AL12" s="2"/>
     </row>
-    <row r="13" spans="1:38" ht="14.25" customHeight="1">
+    <row r="13" spans="1:38" ht="96.6" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="22" t="s">
-        <v>54</v>
+      <c r="B13" s="23" t="s">
+        <v>64</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="9"/>
+      <c r="C13" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>79</v>
+      </c>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="14"/>
+      <c r="J13" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>74</v>
+      </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
@@ -1754,18 +2495,34 @@
       <c r="AK13" s="2"/>
       <c r="AL13" s="2"/>
     </row>
-    <row r="14" spans="1:38" ht="14.25" customHeight="1">
+    <row r="14" spans="1:38" ht="122.4" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="B14" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>106</v>
+      </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -1794,18 +2551,34 @@
       <c r="AK14" s="2"/>
       <c r="AL14" s="2"/>
     </row>
-    <row r="15" spans="1:38" ht="14.25" customHeight="1">
+    <row r="15" spans="1:38" ht="106.8" customHeight="1">
       <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="B15" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>107</v>
+      </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -1834,17 +2607,34 @@
       <c r="AK15" s="2"/>
       <c r="AL15" s="2"/>
     </row>
-    <row r="16" spans="1:38" ht="14.25" customHeight="1">
+    <row r="16" spans="1:38" ht="79.8" customHeight="1">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="B16" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>108</v>
+      </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16" s="2"/>
@@ -1873,18 +2663,34 @@
       <c r="AK16" s="2"/>
       <c r="AL16" s="2"/>
     </row>
-    <row r="17" spans="1:38" ht="14.25" customHeight="1">
+    <row r="17" spans="1:38" ht="79.8" customHeight="1">
       <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="B17" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>109</v>
+      </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
@@ -1913,18 +2719,24 @@
       <c r="AK17" s="2"/>
       <c r="AL17" s="2"/>
     </row>
-    <row r="18" spans="1:38" ht="14.25" customHeight="1">
+    <row r="18" spans="1:38" ht="79.8" customHeight="1">
       <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
+      <c r="B18" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>110</v>
+      </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
@@ -1953,18 +2765,24 @@
       <c r="AK18" s="2"/>
       <c r="AL18" s="2"/>
     </row>
-    <row r="19" spans="1:38" ht="14.25" customHeight="1">
+    <row r="19" spans="1:38" ht="79.8" customHeight="1">
       <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
+      <c r="B19" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K19" s="18" t="s">
+        <v>111</v>
+      </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
@@ -1993,18 +2811,24 @@
       <c r="AK19" s="2"/>
       <c r="AL19" s="2"/>
     </row>
-    <row r="20" spans="1:38" ht="14.25" customHeight="1">
+    <row r="20" spans="1:38" ht="79.8" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
+      <c r="B20" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>112</v>
+      </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -2033,18 +2857,24 @@
       <c r="AK20" s="2"/>
       <c r="AL20" s="2"/>
     </row>
-    <row r="21" spans="1:38" ht="14.25" customHeight="1">
+    <row r="21" spans="1:38" ht="79.8" customHeight="1">
       <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
+      <c r="B21" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K21" s="18" t="s">
+        <v>113</v>
+      </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -2073,18 +2903,24 @@
       <c r="AK21" s="2"/>
       <c r="AL21" s="2"/>
     </row>
-    <row r="22" spans="1:38" ht="14.25" customHeight="1">
+    <row r="22" spans="1:38" ht="79.8" customHeight="1">
       <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
+      <c r="B22" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>114</v>
+      </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
@@ -2115,16 +2951,18 @@
     </row>
     <row r="23" spans="1:38" ht="14.25" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
+      <c r="B23" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="12"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="14"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -2238,7 +3076,6 @@
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -41433,11 +42270,411 @@
       <c r="AK1005" s="2"/>
       <c r="AL1005" s="2"/>
     </row>
+    <row r="1006" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1006" s="2"/>
+      <c r="B1006" s="2"/>
+      <c r="C1006" s="2"/>
+      <c r="D1006" s="3"/>
+      <c r="E1006" s="3"/>
+      <c r="F1006" s="3"/>
+      <c r="G1006" s="2"/>
+      <c r="H1006" s="2"/>
+      <c r="I1006" s="2"/>
+      <c r="J1006" s="2"/>
+      <c r="K1006" s="2"/>
+      <c r="L1006" s="2"/>
+      <c r="M1006" s="2"/>
+      <c r="N1006" s="2"/>
+      <c r="O1006" s="2"/>
+      <c r="P1006" s="2"/>
+      <c r="Q1006" s="2"/>
+      <c r="R1006" s="2"/>
+      <c r="S1006" s="2"/>
+      <c r="T1006" s="2"/>
+      <c r="U1006" s="2"/>
+      <c r="V1006" s="2"/>
+      <c r="W1006" s="2"/>
+      <c r="X1006" s="2"/>
+      <c r="Y1006" s="2"/>
+      <c r="Z1006" s="2"/>
+      <c r="AA1006" s="2"/>
+      <c r="AB1006" s="2"/>
+      <c r="AC1006" s="2"/>
+      <c r="AD1006" s="2"/>
+      <c r="AE1006" s="2"/>
+      <c r="AF1006" s="2"/>
+      <c r="AG1006" s="2"/>
+      <c r="AH1006" s="2"/>
+      <c r="AI1006" s="2"/>
+      <c r="AJ1006" s="2"/>
+      <c r="AK1006" s="2"/>
+      <c r="AL1006" s="2"/>
+    </row>
+    <row r="1007" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1007" s="2"/>
+      <c r="B1007" s="2"/>
+      <c r="C1007" s="2"/>
+      <c r="D1007" s="3"/>
+      <c r="E1007" s="3"/>
+      <c r="F1007" s="3"/>
+      <c r="G1007" s="2"/>
+      <c r="H1007" s="2"/>
+      <c r="I1007" s="2"/>
+      <c r="J1007" s="2"/>
+      <c r="K1007" s="2"/>
+      <c r="L1007" s="2"/>
+      <c r="M1007" s="2"/>
+      <c r="N1007" s="2"/>
+      <c r="O1007" s="2"/>
+      <c r="P1007" s="2"/>
+      <c r="Q1007" s="2"/>
+      <c r="R1007" s="2"/>
+      <c r="S1007" s="2"/>
+      <c r="T1007" s="2"/>
+      <c r="U1007" s="2"/>
+      <c r="V1007" s="2"/>
+      <c r="W1007" s="2"/>
+      <c r="X1007" s="2"/>
+      <c r="Y1007" s="2"/>
+      <c r="Z1007" s="2"/>
+      <c r="AA1007" s="2"/>
+      <c r="AB1007" s="2"/>
+      <c r="AC1007" s="2"/>
+      <c r="AD1007" s="2"/>
+      <c r="AE1007" s="2"/>
+      <c r="AF1007" s="2"/>
+      <c r="AG1007" s="2"/>
+      <c r="AH1007" s="2"/>
+      <c r="AI1007" s="2"/>
+      <c r="AJ1007" s="2"/>
+      <c r="AK1007" s="2"/>
+      <c r="AL1007" s="2"/>
+    </row>
+    <row r="1008" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1008" s="2"/>
+      <c r="B1008" s="2"/>
+      <c r="C1008" s="2"/>
+      <c r="D1008" s="3"/>
+      <c r="E1008" s="3"/>
+      <c r="F1008" s="3"/>
+      <c r="G1008" s="2"/>
+      <c r="H1008" s="2"/>
+      <c r="I1008" s="2"/>
+      <c r="J1008" s="2"/>
+      <c r="K1008" s="2"/>
+      <c r="L1008" s="2"/>
+      <c r="M1008" s="2"/>
+      <c r="N1008" s="2"/>
+      <c r="O1008" s="2"/>
+      <c r="P1008" s="2"/>
+      <c r="Q1008" s="2"/>
+      <c r="R1008" s="2"/>
+      <c r="S1008" s="2"/>
+      <c r="T1008" s="2"/>
+      <c r="U1008" s="2"/>
+      <c r="V1008" s="2"/>
+      <c r="W1008" s="2"/>
+      <c r="X1008" s="2"/>
+      <c r="Y1008" s="2"/>
+      <c r="Z1008" s="2"/>
+      <c r="AA1008" s="2"/>
+      <c r="AB1008" s="2"/>
+      <c r="AC1008" s="2"/>
+      <c r="AD1008" s="2"/>
+      <c r="AE1008" s="2"/>
+      <c r="AF1008" s="2"/>
+      <c r="AG1008" s="2"/>
+      <c r="AH1008" s="2"/>
+      <c r="AI1008" s="2"/>
+      <c r="AJ1008" s="2"/>
+      <c r="AK1008" s="2"/>
+      <c r="AL1008" s="2"/>
+    </row>
+    <row r="1009" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1009" s="2"/>
+      <c r="B1009" s="2"/>
+      <c r="C1009" s="2"/>
+      <c r="D1009" s="3"/>
+      <c r="E1009" s="3"/>
+      <c r="F1009" s="3"/>
+      <c r="G1009" s="2"/>
+      <c r="H1009" s="2"/>
+      <c r="I1009" s="2"/>
+      <c r="J1009" s="2"/>
+      <c r="K1009" s="2"/>
+      <c r="L1009" s="2"/>
+      <c r="M1009" s="2"/>
+      <c r="N1009" s="2"/>
+      <c r="O1009" s="2"/>
+      <c r="P1009" s="2"/>
+      <c r="Q1009" s="2"/>
+      <c r="R1009" s="2"/>
+      <c r="S1009" s="2"/>
+      <c r="T1009" s="2"/>
+      <c r="U1009" s="2"/>
+      <c r="V1009" s="2"/>
+      <c r="W1009" s="2"/>
+      <c r="X1009" s="2"/>
+      <c r="Y1009" s="2"/>
+      <c r="Z1009" s="2"/>
+      <c r="AA1009" s="2"/>
+      <c r="AB1009" s="2"/>
+      <c r="AC1009" s="2"/>
+      <c r="AD1009" s="2"/>
+      <c r="AE1009" s="2"/>
+      <c r="AF1009" s="2"/>
+      <c r="AG1009" s="2"/>
+      <c r="AH1009" s="2"/>
+      <c r="AI1009" s="2"/>
+      <c r="AJ1009" s="2"/>
+      <c r="AK1009" s="2"/>
+      <c r="AL1009" s="2"/>
+    </row>
+    <row r="1010" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1010" s="2"/>
+      <c r="B1010" s="2"/>
+      <c r="C1010" s="2"/>
+      <c r="D1010" s="3"/>
+      <c r="E1010" s="3"/>
+      <c r="F1010" s="3"/>
+      <c r="G1010" s="2"/>
+      <c r="H1010" s="2"/>
+      <c r="I1010" s="2"/>
+      <c r="J1010" s="2"/>
+      <c r="K1010" s="2"/>
+      <c r="L1010" s="2"/>
+      <c r="M1010" s="2"/>
+      <c r="N1010" s="2"/>
+      <c r="O1010" s="2"/>
+      <c r="P1010" s="2"/>
+      <c r="Q1010" s="2"/>
+      <c r="R1010" s="2"/>
+      <c r="S1010" s="2"/>
+      <c r="T1010" s="2"/>
+      <c r="U1010" s="2"/>
+      <c r="V1010" s="2"/>
+      <c r="W1010" s="2"/>
+      <c r="X1010" s="2"/>
+      <c r="Y1010" s="2"/>
+      <c r="Z1010" s="2"/>
+      <c r="AA1010" s="2"/>
+      <c r="AB1010" s="2"/>
+      <c r="AC1010" s="2"/>
+      <c r="AD1010" s="2"/>
+      <c r="AE1010" s="2"/>
+      <c r="AF1010" s="2"/>
+      <c r="AG1010" s="2"/>
+      <c r="AH1010" s="2"/>
+      <c r="AI1010" s="2"/>
+      <c r="AJ1010" s="2"/>
+      <c r="AK1010" s="2"/>
+      <c r="AL1010" s="2"/>
+    </row>
+    <row r="1011" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1011" s="2"/>
+      <c r="B1011" s="2"/>
+      <c r="C1011" s="2"/>
+      <c r="D1011" s="3"/>
+      <c r="E1011" s="3"/>
+      <c r="F1011" s="3"/>
+      <c r="G1011" s="2"/>
+      <c r="H1011" s="2"/>
+      <c r="I1011" s="2"/>
+      <c r="J1011" s="2"/>
+      <c r="K1011" s="2"/>
+      <c r="L1011" s="2"/>
+      <c r="M1011" s="2"/>
+      <c r="N1011" s="2"/>
+      <c r="O1011" s="2"/>
+      <c r="P1011" s="2"/>
+      <c r="Q1011" s="2"/>
+      <c r="R1011" s="2"/>
+      <c r="S1011" s="2"/>
+      <c r="T1011" s="2"/>
+      <c r="U1011" s="2"/>
+      <c r="V1011" s="2"/>
+      <c r="W1011" s="2"/>
+      <c r="X1011" s="2"/>
+      <c r="Y1011" s="2"/>
+      <c r="Z1011" s="2"/>
+      <c r="AA1011" s="2"/>
+      <c r="AB1011" s="2"/>
+      <c r="AC1011" s="2"/>
+      <c r="AD1011" s="2"/>
+      <c r="AE1011" s="2"/>
+      <c r="AF1011" s="2"/>
+      <c r="AG1011" s="2"/>
+      <c r="AH1011" s="2"/>
+      <c r="AI1011" s="2"/>
+      <c r="AJ1011" s="2"/>
+      <c r="AK1011" s="2"/>
+      <c r="AL1011" s="2"/>
+    </row>
+    <row r="1012" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1012" s="2"/>
+      <c r="B1012" s="2"/>
+      <c r="C1012" s="2"/>
+      <c r="D1012" s="3"/>
+      <c r="E1012" s="3"/>
+      <c r="F1012" s="3"/>
+      <c r="G1012" s="2"/>
+      <c r="H1012" s="2"/>
+      <c r="I1012" s="2"/>
+      <c r="J1012" s="2"/>
+      <c r="K1012" s="2"/>
+      <c r="L1012" s="2"/>
+      <c r="M1012" s="2"/>
+      <c r="N1012" s="2"/>
+      <c r="O1012" s="2"/>
+      <c r="P1012" s="2"/>
+      <c r="Q1012" s="2"/>
+      <c r="R1012" s="2"/>
+      <c r="S1012" s="2"/>
+      <c r="T1012" s="2"/>
+      <c r="U1012" s="2"/>
+      <c r="V1012" s="2"/>
+      <c r="W1012" s="2"/>
+      <c r="X1012" s="2"/>
+      <c r="Y1012" s="2"/>
+      <c r="Z1012" s="2"/>
+      <c r="AA1012" s="2"/>
+      <c r="AB1012" s="2"/>
+      <c r="AC1012" s="2"/>
+      <c r="AD1012" s="2"/>
+      <c r="AE1012" s="2"/>
+      <c r="AF1012" s="2"/>
+      <c r="AG1012" s="2"/>
+      <c r="AH1012" s="2"/>
+      <c r="AI1012" s="2"/>
+      <c r="AJ1012" s="2"/>
+      <c r="AK1012" s="2"/>
+      <c r="AL1012" s="2"/>
+    </row>
+    <row r="1013" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1013" s="2"/>
+      <c r="B1013" s="2"/>
+      <c r="C1013" s="2"/>
+      <c r="D1013" s="3"/>
+      <c r="E1013" s="3"/>
+      <c r="F1013" s="3"/>
+      <c r="G1013" s="2"/>
+      <c r="H1013" s="2"/>
+      <c r="I1013" s="2"/>
+      <c r="J1013" s="2"/>
+      <c r="K1013" s="2"/>
+      <c r="L1013" s="2"/>
+      <c r="M1013" s="2"/>
+      <c r="N1013" s="2"/>
+      <c r="O1013" s="2"/>
+      <c r="P1013" s="2"/>
+      <c r="Q1013" s="2"/>
+      <c r="R1013" s="2"/>
+      <c r="S1013" s="2"/>
+      <c r="T1013" s="2"/>
+      <c r="U1013" s="2"/>
+      <c r="V1013" s="2"/>
+      <c r="W1013" s="2"/>
+      <c r="X1013" s="2"/>
+      <c r="Y1013" s="2"/>
+      <c r="Z1013" s="2"/>
+      <c r="AA1013" s="2"/>
+      <c r="AB1013" s="2"/>
+      <c r="AC1013" s="2"/>
+      <c r="AD1013" s="2"/>
+      <c r="AE1013" s="2"/>
+      <c r="AF1013" s="2"/>
+      <c r="AG1013" s="2"/>
+      <c r="AH1013" s="2"/>
+      <c r="AI1013" s="2"/>
+      <c r="AJ1013" s="2"/>
+      <c r="AK1013" s="2"/>
+      <c r="AL1013" s="2"/>
+    </row>
+    <row r="1014" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1014" s="2"/>
+      <c r="B1014" s="2"/>
+      <c r="C1014" s="2"/>
+      <c r="D1014" s="3"/>
+      <c r="E1014" s="3"/>
+      <c r="F1014" s="3"/>
+      <c r="G1014" s="2"/>
+      <c r="H1014" s="2"/>
+      <c r="I1014" s="2"/>
+      <c r="J1014" s="2"/>
+      <c r="K1014" s="2"/>
+      <c r="L1014" s="2"/>
+      <c r="M1014" s="2"/>
+      <c r="N1014" s="2"/>
+      <c r="O1014" s="2"/>
+      <c r="P1014" s="2"/>
+      <c r="Q1014" s="2"/>
+      <c r="R1014" s="2"/>
+      <c r="S1014" s="2"/>
+      <c r="T1014" s="2"/>
+      <c r="U1014" s="2"/>
+      <c r="V1014" s="2"/>
+      <c r="W1014" s="2"/>
+      <c r="X1014" s="2"/>
+      <c r="Y1014" s="2"/>
+      <c r="Z1014" s="2"/>
+      <c r="AA1014" s="2"/>
+      <c r="AB1014" s="2"/>
+      <c r="AC1014" s="2"/>
+      <c r="AD1014" s="2"/>
+      <c r="AE1014" s="2"/>
+      <c r="AF1014" s="2"/>
+      <c r="AG1014" s="2"/>
+      <c r="AH1014" s="2"/>
+      <c r="AI1014" s="2"/>
+      <c r="AJ1014" s="2"/>
+      <c r="AK1014" s="2"/>
+      <c r="AL1014" s="2"/>
+    </row>
+    <row r="1015" spans="1:38" ht="14.25" customHeight="1">
+      <c r="A1015" s="2"/>
+      <c r="B1015" s="2"/>
+      <c r="C1015" s="2"/>
+      <c r="D1015" s="3"/>
+      <c r="E1015" s="3"/>
+      <c r="F1015" s="3"/>
+      <c r="G1015" s="2"/>
+      <c r="H1015" s="2"/>
+      <c r="I1015" s="2"/>
+      <c r="J1015" s="2"/>
+      <c r="K1015" s="2"/>
+      <c r="L1015" s="2"/>
+      <c r="M1015" s="2"/>
+      <c r="N1015" s="2"/>
+      <c r="O1015" s="2"/>
+      <c r="P1015" s="2"/>
+      <c r="Q1015" s="2"/>
+      <c r="R1015" s="2"/>
+      <c r="S1015" s="2"/>
+      <c r="T1015" s="2"/>
+      <c r="U1015" s="2"/>
+      <c r="V1015" s="2"/>
+      <c r="W1015" s="2"/>
+      <c r="X1015" s="2"/>
+      <c r="Y1015" s="2"/>
+      <c r="Z1015" s="2"/>
+      <c r="AA1015" s="2"/>
+      <c r="AB1015" s="2"/>
+      <c r="AC1015" s="2"/>
+      <c r="AD1015" s="2"/>
+      <c r="AE1015" s="2"/>
+      <c r="AF1015" s="2"/>
+      <c r="AG1015" s="2"/>
+      <c r="AH1015" s="2"/>
+      <c r="AI1015" s="2"/>
+      <c r="AJ1015" s="2"/>
+      <c r="AK1015" s="2"/>
+      <c r="AL1015" s="2"/>
+    </row>
   </sheetData>
   <customSheetViews>
     <customSheetView guid="{594E70F7-1077-448A-A0CF-FD3289E530C0}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="B2:K8" xr:uid="{0BB350B9-66AB-4DC9-966C-1DB8FE3D1FE4}"/>
+      <autoFilter ref="B2:K8" xr:uid="{CEDE2193-D922-4B49-81E1-2F0077F859D1}"/>
       <extLst>
         <ext uri="GoogleSheetsCustomDataVersion1">
           <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" filterViewId="268527203"/>
@@ -41445,7 +42682,8 @@
       </extLst>
     </customSheetView>
   </customSheetViews>
-  <conditionalFormatting sqref="J3:J13">
+  <phoneticPr fontId="10" type="noConversion"/>
+  <conditionalFormatting sqref="J3:J23">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>$AL$5</formula>
     </cfRule>
@@ -41454,7 +42692,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J3:J13" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J3:J23" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$AL$1:$AL$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -41466,8 +42704,18 @@
     <hyperlink ref="K8" location="TC_05!A1" display="TC_05!A1" xr:uid="{760CBD34-0C80-45D2-933E-3E1EF10F2C8D}"/>
     <hyperlink ref="K9" location="TC_06!A1" display="TC_06!A1" xr:uid="{97927EEC-4CB6-43C8-9D30-217CE36B494C}"/>
     <hyperlink ref="K10" location="TC_07!A1" display="TC_07!A1" xr:uid="{57761202-4B5A-4794-8C37-021A847C2891}"/>
+    <hyperlink ref="K22" location="TC_19!A1" display="TC_19!A1" xr:uid="{5B637FC8-B887-4E54-A734-3410ACD58EE2}"/>
     <hyperlink ref="K11" location="TC_08!A1" display="TC_08!A1" xr:uid="{8DCDCBB1-F1F9-42E4-8738-B4AAD74C393D}"/>
-    <hyperlink ref="K12" location="TC_09!A1" display="TC_09!A1" xr:uid="{5B637FC8-B887-4E54-A734-3410ACD58EE2}"/>
+    <hyperlink ref="K12:K21" location="TC_09!A1" display="TC_09!A1" xr:uid="{02F14F77-9FA9-4814-A813-BFCACA6D631D}"/>
+    <hyperlink ref="K13" location="TC_10!A1" display="TC_10!A1" xr:uid="{FF168EAB-26B6-4FD3-9BC1-40D2CDE56290}"/>
+    <hyperlink ref="K14" location="TC_11!A1" display="TC_11!A1" xr:uid="{02C55C44-A99B-4932-8DAA-25C59D1B4BC8}"/>
+    <hyperlink ref="K15" location="TC_12!A1" display="TC_12!A1" xr:uid="{0AD2F14D-FEEB-49C0-8F4E-E282E69B32C8}"/>
+    <hyperlink ref="K16" location="TC_13!A1" display="TC_13!A1" xr:uid="{E100C207-D52F-4B3B-ACA0-966D3B6C9B72}"/>
+    <hyperlink ref="K17" location="TC_14!A1" display="TC_14!A1" xr:uid="{1D74BB79-3A89-4CD2-828A-5178BB70BA27}"/>
+    <hyperlink ref="K18" location="TC_15!A1" display="TC_15!A1" xr:uid="{297E2164-CE07-4E16-8DD9-77FEFC124AE3}"/>
+    <hyperlink ref="K19" location="TC_16!A1" display="TC_16!A1" xr:uid="{B4A79609-5555-44F6-A4A1-25CA4F1DB939}"/>
+    <hyperlink ref="K20" location="TC_17!A1" display="TC_17!A1" xr:uid="{31110212-2A34-47CB-9C5D-BDE91564333B}"/>
+    <hyperlink ref="K21" location="TC_18!A1" display="TC_18!A1" xr:uid="{F1E8B5F0-EFB3-48E8-93C0-3D5D0EFC0AAE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -41485,6 +42733,147 @@
     <row r="2" spans="2:2">
       <c r="B2" s="19" t="s">
         <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2018B9FA-72E4-4773-984A-8F7D1FE87592}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51BE4F90-C957-4F9A-9C0A-1BB2D735BF47}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05AD05E-7BB6-4108-B1D7-FCAECB9A3DBF}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30C9B434-52CA-48AA-8AC7-BC977CEFC06A}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3DCFD27-C8D7-4A2B-8C17-6AF6BA6229C0}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F9E749A-60F8-48F5-ABB9-99D697D8B6E6}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E8EF50-A4A6-4AC4-9A2D-11EC3A2821B1}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2B1521E-5647-40C5-9D06-AF9184D31439}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0BFB99C-BCA4-4A3B-A397-53A2A1FCCA32}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -42512,6 +43901,51 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{765A5931-DB83-472E-9C62-5D069DAB698B}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B06AC935-6278-4DCF-B55A-62855BFE8DEA}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3707936-371D-4EC4-9209-02DC8F0591A0}">
+  <dimension ref="B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="2" spans="2:2">
+      <c r="B2" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -44605,6 +46039,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -44620,6 +46055,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -44635,5 +46071,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>